<commit_message>
hb data 2025 processed
</commit_message>
<xml_diff>
--- a/data/hb/original_data/apc_hb_2025.xlsx
+++ b/data/hb/original_data/apc_hb_2025.xlsx
@@ -1,16 +1,16 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29825"/>
+  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="10328"/>
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="https://boras-my.sharepoint.com/personal/signe_wulund_hb_se/Documents/Rapporter, sammanställningar mm/"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="/Users/2021m30/R/repos/openapc-se/data/hb/original_data/"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="1" documentId="8_{5E3139A5-6079-4766-A1B3-B663A63C5711}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{443B294C-E41C-4C35-AD6C-67EB197F83D4}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="8_{D9ABD2C9-DF70-F34D-8252-616175F29DCC}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="17640" xr2:uid="{F788AA10-277E-44C1-A5DB-D859C87D55A3}"/>
+    <workbookView xWindow="-120" yWindow="600" windowWidth="29040" windowHeight="17640" xr2:uid="{F788AA10-277E-44C1-A5DB-D859C87D55A3}"/>
   </bookViews>
   <sheets>
     <sheet name="apc_template" sheetId="2" r:id="rId1"/>
@@ -20,6 +20,7 @@
     <definedName name="ExternalData_1" localSheetId="0" hidden="1">apc_template!$A$1:$K$1</definedName>
   </definedNames>
   <calcPr calcId="191028"/>
+  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -102,7 +103,7 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="1">
+  <fonts count="1" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -138,44 +139,7 @@
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
   </cellStyles>
-  <dxfs count="12">
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-    <dxf>
-      <numFmt numFmtId="0" formatCode="General"/>
-    </dxf>
-  </dxfs>
+  <dxfs count="0"/>
   <tableStyles count="0" defaultTableStyle="TableStyleMedium2" defaultPivotStyle="PivotStyleLight16"/>
   <extLst>
     <ext xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" uri="{EB79DEF2-80B8-43e5-95BD-54CBDDF9020C}">
@@ -186,46 +150,6 @@
     </ext>
   </extLst>
 </styleSheet>
-</file>
-
-<file path=xl/queryTables/queryTable1.xml><?xml version="1.0" encoding="utf-8"?>
-<queryTable xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr16="http://schemas.microsoft.com/office/spreadsheetml/2017/revision16" mc:Ignorable="xr16" name="ExternalData_1" connectionId="1" xr16:uid="{01CF655A-704F-40D2-877F-6968F7CA8292}" autoFormatId="16" applyNumberFormats="0" applyBorderFormats="0" applyFontFormats="0" applyPatternFormats="0" applyAlignmentFormats="0" applyWidthHeightFormats="0">
-  <queryTableRefresh nextId="12">
-    <queryTableFields count="11">
-      <queryTableField id="1" name="Column1" tableColumnId="1"/>
-      <queryTableField id="2" name="Column2" tableColumnId="2"/>
-      <queryTableField id="3" name="Column3" tableColumnId="3"/>
-      <queryTableField id="4" name="Column4" tableColumnId="4"/>
-      <queryTableField id="5" name="Column5" tableColumnId="5"/>
-      <queryTableField id="6" name="Column6" tableColumnId="6"/>
-      <queryTableField id="7" name="Column7" tableColumnId="7"/>
-      <queryTableField id="8" name="Column8" tableColumnId="8"/>
-      <queryTableField id="9" name="Column9" tableColumnId="9"/>
-      <queryTableField id="10" name="Column10" tableColumnId="10"/>
-      <queryTableField id="11" name="Column11" tableColumnId="11"/>
-    </queryTableFields>
-  </queryTableRefresh>
-</queryTable>
-</file>
-
-<file path=xl/tables/table1.xml><?xml version="1.0" encoding="utf-8"?>
-<table xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="xr xr3" id="1" xr:uid="{251F5501-7CAD-4CB9-BEBB-61320C7E10B0}" name="apc_template" displayName="apc_template" ref="A1:K4" tableType="queryTable" totalsRowShown="0" headerRowDxfId="11">
-  <autoFilter ref="A1:K4" xr:uid="{251F5501-7CAD-4CB9-BEBB-61320C7E10B0}"/>
-  <tableColumns count="11">
-    <tableColumn id="1" xr3:uid="{75808B81-283D-4AFA-B8B5-2F47F238B0E8}" uniqueName="1" name="institution" queryTableFieldId="1" dataDxfId="10"/>
-    <tableColumn id="2" xr3:uid="{2996A03E-6D52-4DA4-AD4F-3C0D81D3BADF}" uniqueName="2" name="period" queryTableFieldId="2" dataDxfId="9"/>
-    <tableColumn id="3" xr3:uid="{AA6657BC-A523-4815-B0D1-DC1EAF8E7307}" uniqueName="3" name="sek" queryTableFieldId="3" dataDxfId="8"/>
-    <tableColumn id="4" xr3:uid="{E2C030DF-9E5C-49D9-B9DA-F992BEAA0EC9}" uniqueName="4" name="doi" queryTableFieldId="4" dataDxfId="7"/>
-    <tableColumn id="5" xr3:uid="{B940954B-F125-43AE-8D12-F9DCC147EEA9}" uniqueName="5" name="is_hybrid" queryTableFieldId="5" dataDxfId="6"/>
-    <tableColumn id="6" xr3:uid="{5A737D0C-1428-4DEC-B9A1-2AF3921B91BD}" uniqueName="6" name="publisher" queryTableFieldId="6" dataDxfId="5"/>
-    <tableColumn id="7" xr3:uid="{B146D14B-1308-4CAF-A328-B6048BA47A9C}" uniqueName="7" name="journal_full_title" queryTableFieldId="7" dataDxfId="4"/>
-    <tableColumn id="8" xr3:uid="{2841498F-B502-4D2B-8210-82B06B1BF552}" uniqueName="8" name="issn" queryTableFieldId="8" dataDxfId="3"/>
-    <tableColumn id="9" xr3:uid="{E6EEB2CB-F7B1-4987-BB05-3EFC1BA0EE30}" uniqueName="9" name="issn_print" queryTableFieldId="9" dataDxfId="2"/>
-    <tableColumn id="10" xr3:uid="{8027D1B9-8D9D-4C28-BEEA-9BF7A71C1D68}" uniqueName="10" name="issn_electronic" queryTableFieldId="10" dataDxfId="1"/>
-    <tableColumn id="11" xr3:uid="{1FECB6C9-0985-467A-A5FC-74FBFD9D61B0}" uniqueName="11" name="url" queryTableFieldId="11" dataDxfId="0"/>
-  </tableColumns>
-  <tableStyleInfo name="TableStyleMedium7" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
-</table>
 </file>
 
 <file path=xl/theme/theme1.xml><?xml version="1.0" encoding="utf-8"?>
@@ -546,18 +470,18 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{48DB2F83-4BFA-47BD-A67A-72BCD144BC37}">
   <dimension ref="A1:K4"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <cols>
-    <col min="1" max="5" width="10.7109375" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="11.140625" bestFit="1" customWidth="1"/>
-    <col min="7" max="7" width="16.7109375" bestFit="1" customWidth="1"/>
-    <col min="8" max="8" width="6.5703125" bestFit="1" customWidth="1"/>
-    <col min="9" max="9" width="11.28515625" bestFit="1" customWidth="1"/>
-    <col min="10" max="10" width="15.85546875" bestFit="1" customWidth="1"/>
-    <col min="11" max="11" width="5.42578125" bestFit="1" customWidth="1"/>
+    <col min="1" max="5" width="10.6640625" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="11.1640625" bestFit="1" customWidth="1"/>
+    <col min="7" max="7" width="16.6640625" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="6.5" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="11.33203125" bestFit="1" customWidth="1"/>
+    <col min="10" max="10" width="15.83203125" bestFit="1" customWidth="1"/>
+    <col min="11" max="11" width="5.5" bestFit="1" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:11">
+    <row r="1" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A1" t="s">
         <v>0</v>
       </c>
@@ -592,7 +516,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="2" spans="1:11">
+    <row r="2" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A2" t="s">
         <v>11</v>
       </c>
@@ -609,7 +533,7 @@
         <v>1</v>
       </c>
     </row>
-    <row r="3" spans="1:11">
+    <row r="3" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A3" t="s">
         <v>11</v>
       </c>
@@ -626,7 +550,7 @@
         <v>0</v>
       </c>
     </row>
-    <row r="4" spans="1:11">
+    <row r="4" spans="1:11" x14ac:dyDescent="0.2">
       <c r="A4" t="s">
         <v>11</v>
       </c>
@@ -645,16 +569,13 @@
     </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
-  <tableParts count="1">
-    <tablePart r:id="rId1"/>
-  </tableParts>
 </worksheet>
 </file>
 
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{19E8F8B7-E035-4372-AB95-74A11E49D8E1}">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.45"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="8.83203125" defaultRowHeight="15" x14ac:dyDescent="0.2"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
@@ -664,5 +585,9 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFC8AC1D-F7E8-4D23-BBAB-985BA9072E2D}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{DFC8AC1D-F7E8-4D23-BBAB-985BA9072E2D}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/DataMashup"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
 </file>
</xml_diff>